<commit_message>
Track D-022 as an open documentation update
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AzN61zWTi2yq5SJaQMPbTS
</commit_message>
<xml_diff>
--- a/docs/BEST_Document_Alignment_Tracker.xlsx
+++ b/docs/BEST_Document_Alignment_Tracker.xlsx
@@ -55,7 +55,7 @@
       <sz val="10.5"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -92,6 +92,11 @@
         <fgColor rgb="00E3F5EC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -110,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,6 +141,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1170,7 +1178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2143,9 +2151,44 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Platform master data (D-022)</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Not in PRD v3.1, catalogue or schema</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Consent items, assessment types and validity, client profiles, checklist library, devices, signal parameters, reason lists, client fields</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>D-022, 28 Oct</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>Needs decision</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Kept open by Sujit: PRD §8.12, §8.13; catalogue (3 new permissions); schema (new collections)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Agreed,Agreed in review,Agreed internally,Awaiting client,Pending client,Needs decision"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
MongoDB schema extended with D-022 platform master data (26 collections)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AzN61zWTi2yq5SJaQMPbTS
</commit_message>
<xml_diff>
--- a/docs/BEST_Document_Alignment_Tracker.xlsx
+++ b/docs/BEST_Document_Alignment_Tracker.xlsx
@@ -984,7 +984,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>MongoDB schema (user creation)</t>
+          <t>MongoDB schema</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1004,12 +1004,12 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>13 collections for user creation and login</t>
+          <t>26 collections: user creation and login (13) and platform master data (13, D-022)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Follows role-first and D-019</t>
+          <t>Follows D-019, D-021, D-022</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Kept open by Sujit: PRD §8.12, §8.13; catalogue (3 new permissions); schema (new collections)</t>
+          <t>In the schema (28 Oct). Still open: PRD §8.12, §8.13; catalogue and FSD §2.2 (3 new Clinic settings permissions: checklists, reason lists, client fields)</t>
         </is>
       </c>
     </row>

</xml_diff>